<commit_message>
Restore real cleavable scan 2, switch plots to linear interpolation
Replaces the empty cleavable scan 2 export with the real data from
Max's own archive (previously shown as missing), and corrects its
time to 8 min (was assumed to be 5 min). Drops LOWESS smoothing
entirely per Max's request: all trend lines are now plain straight-
line interpolation between the real, included points, nothing
estimated. Retitles the figures to "20 nM MMP-9 SWV Measurements, 60
Minutes -- <condition>". Regenerates the peak data export and the
zip for Max accordingly.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/electrochemical_device/models/11_swv_forward/max_peaks_figures/max_peaks_data.xlsx
+++ b/electrochemical_device/models/11_swv_forward/max_peaks_figures/max_peaks_data.xlsx
@@ -439,7 +439,7 @@
     <col width="20" customWidth="1" min="10" max="10"/>
     <col width="13" customWidth="1" min="11" max="11"/>
     <col width="16" customWidth="1" min="12" max="12"/>
-    <col width="29" customWidth="1" min="13" max="13"/>
+    <col width="7" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -578,11 +578,47 @@
         <v>2</v>
       </c>
       <c r="B6" t="n">
-        <v>5</v>
+        <v>8</v>
+      </c>
+      <c r="C6" t="n">
+        <v>9.673999999999999</v>
+      </c>
+      <c r="D6" t="n">
+        <v>-244.1</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>62.2</v>
+      </c>
+      <c r="G6" t="n">
+        <v>8.449999999999999</v>
+      </c>
+      <c r="H6" t="n">
+        <v>289.5</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="J6" t="n">
+        <v>49.1</v>
+      </c>
+      <c r="K6" t="n">
+        <v>1.145</v>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>missing: empty .xlsx export</t>
+          <t>ok</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Restore real BSA control scans 2, 3 and 11
These three were empty .xlsx exports (0 bytes); replaced with the
real data from Max's own archive. All 13 BSA control scans are now
present. Regenerates the BSA signal-vs-time plot and the peak data
export/zip accordingly.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/electrochemical_device/models/11_swv_forward/max_peaks_figures/max_peaks_data.xlsx
+++ b/electrochemical_device/models/11_swv_forward/max_peaks_figures/max_peaks_data.xlsx
@@ -2004,9 +2004,18 @@
       <c r="B6" t="n">
         <v>5</v>
       </c>
+      <c r="C6" t="n">
+        <v>339.386</v>
+      </c>
+      <c r="D6" t="n">
+        <v>59.8</v>
+      </c>
+      <c r="E6" t="n">
+        <v>93.2</v>
+      </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>missing: empty .xlsx export</t>
+          <t>not MB or Fc (outside both their windows); real local peak, -50 to +150 mV window</t>
         </is>
       </c>
     </row>
@@ -2017,9 +2026,18 @@
       <c r="B7" t="n">
         <v>10</v>
       </c>
+      <c r="C7" t="n">
+        <v>252.38</v>
+      </c>
+      <c r="D7" t="n">
+        <v>75.7</v>
+      </c>
+      <c r="E7" t="n">
+        <v>69.3</v>
+      </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>missing: empty .xlsx export</t>
+          <t>not MB or Fc (outside both their windows); real local peak, -50 to +150 mV window</t>
         </is>
       </c>
     </row>
@@ -2184,9 +2202,18 @@
       <c r="B15" t="n">
         <v>50</v>
       </c>
+      <c r="C15" t="n">
+        <v>268.86</v>
+      </c>
+      <c r="D15" t="n">
+        <v>75.7</v>
+      </c>
+      <c r="E15" t="n">
+        <v>73.8</v>
+      </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>missing: empty .xlsx export</t>
+          <t>not MB or Fc (outside both their windows); real local peak, -50 to +150 mV window</t>
         </is>
       </c>
     </row>

</xml_diff>